<commit_message>
Update feifeng-wangong-xlsx 2026-10-14 10:02
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -545,11 +545,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 06:17:17</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -598,17 +598,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196312</t>
+          <t>C01310018</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>小齿轮轴</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -616,7 +616,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>渗透探伤（PT）</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,7 +626,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-26 16:19:07</t>
+          <t>2026-09-08 03:17:49</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -636,25 +641,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300218</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>主齿轮</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -664,22 +669,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-06 13:59:23</t>
+          <t>2026-10-13 13:04:07</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01310018</t>
+          <t>C05000066</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>花键法兰</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -688,11 +693,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>倒角</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -702,27 +707,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17:49</t>
+          <t>2026-10-09 10:40:27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C05000066</t>
+          <t>C05000014</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>花键法兰</t>
+          <t>法兰</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -731,30 +736,30 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>倒角</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-09 10:40:38</t>
+          <t>2026-10-09 17:18:09</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-11-05 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -803,25 +808,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01196359</t>
+          <t>C01196296</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>一二级高速轴</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,17 +836,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-28 16:52:31</t>
+          <t>2026-10-13 13:39:35</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196363</t>
+          <t>C01196359</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -851,7 +856,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -859,7 +864,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -869,12 +874,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-06 10:42:15</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-09-28 16:52:31</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -965,12 +965,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01166011</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>消隙直齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -979,11 +979,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -993,27 +993,27 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-15 15:47:08</t>
+          <t>2026-10-12 10:59:11</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-01 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01176035</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>二级消隙齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1022,11 +1022,11 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1036,27 +1036,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-12 11:12:30</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-11-20 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XY06110</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>输出行星轮</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>超精磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1079,48 +1079,96 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2025-04-17 10:57:01</t>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-11-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>3</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-09-27 07:59:31</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1135,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1313,25 +1361,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C14006237</t>
+          <t>C01310070</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>外套</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1341,19 +1389,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-12 13:02:07</t>
+          <t>2026-10-13 20:25:16</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C14006237</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1362,11 +1415,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1376,32 +1429,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-27 13:59:36</t>
+          <t>2026-10-12 13:02:07</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1411,72 +1464,67 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-13 15:21:27</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C05000014</t>
+          <t>C01300218</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>法兰</t>
+          <t>主齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-09 17:18:09</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-11-05 00:00:00</t>
+          <t>2026-10-06 13:59:23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>C01310054</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1486,37 +1534,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-07-27 13:59:36</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01176035</t>
+          <t>C07000124</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>二级消隙齿轮</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1526,50 +1569,85 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 11:12:30</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-12 23:10:08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>C01300223</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>大齿轮组件</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>动平衡</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:54:55</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>CC092679</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>3</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>加工中心</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>2026-06-03 14:50:03</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1586,7 +1664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1650,7 +1728,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1664,11 +1742,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>加工中心2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1678,7 +1756,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-11 01:37:19</t>
+          <t>2026-10-13 15:55:41</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1690,7 +1768,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1704,7 +1782,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1718,42 +1796,37 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-10 15:16:19</t>
+          <t>2026-10-11 01:37:19</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>磁粉探伤-退磁</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300491</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1763,37 +1836,42 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-29 09:19:29</t>
+          <t>2026-10-10 15:16:19</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1803,24 +1881,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-12 10:11:54</t>
+          <t>2026-10-13 10:55:27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196296</t>
+          <t>C01300491</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1829,11 +1912,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1843,7 +1926,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-08 18:41:49</t>
+          <t>2026-09-29 09:19:29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1894,6 +1977,46 @@
       <c r="I7" t="inlineStr">
         <is>
           <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C01300253</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>齿轮（左）</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-13 18:17:38</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-15 08:53
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,25 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C07000138</t>
+          <t>C01300202</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>轮轴#</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,27 +507,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-28 10:57:42</t>
+          <t>2026-10-11 12:55:33</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196210</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮轴组件</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -535,7 +540,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>检测</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -545,7 +550,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-14 10:26:31</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -555,12 +565,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300202</t>
+          <t>C01310018</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -569,11 +579,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -583,27 +593,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-11 12:55:33</t>
+          <t>2026-09-08 03:17:49</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01310018</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -612,11 +622,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,27 +636,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17:49</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-13 13:04:07</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C05000014</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>法兰</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -655,36 +660,41 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-13 13:04:07</t>
+          <t>2026-10-09 17:18:09</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-11-05 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C05000066</t>
+          <t>C01300541</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>花键法兰</t>
+          <t>Z326M6齿圈</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -693,11 +703,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>倒角</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -707,12 +717,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-09 10:40:27</t>
+          <t>2026-10-10 16:02:04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -722,17 +732,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C05000014</t>
+          <t>C01196296</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>法兰</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -740,22 +750,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-09 17:18:09</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-11-05 00:00:00</t>
+          <t>2026-10-13 13:39:35</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -765,17 +770,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>CC090887</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -783,7 +788,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -793,40 +798,40 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
+          <t>2026-10-12 13:59:57</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01196296</t>
+          <t>CC090888</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -836,35 +841,35 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-13 13:39:35</t>
+          <t>2026-10-12 13:59:28</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196359</t>
+          <t>C01166011</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>一二级高速轴</t>
+          <t>消隙直齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -874,35 +879,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-28 16:52:31</t>
+          <t>2026-10-12 10:59:11</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CC090887</t>
+          <t>C01176035</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>二级消隙齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -912,40 +922,40 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:57</t>
+          <t>2026-10-12 11:12:30</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -955,22 +965,27 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:28</t>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -979,11 +994,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -993,27 +1008,27 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-11-20 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01176035</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>二级消隙齿轮</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1022,11 +1037,11 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1036,139 +1051,10 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-12 11:12:30</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1183,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1401,21 +1287,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C14006237</t>
+          <t>C01300491</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1429,19 +1315,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-12 13:02:07</t>
+          <t>2026-10-14 18:05:38</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1450,11 +1336,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1464,32 +1350,37 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-13 17:54:55</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300218</t>
+          <t>C01196390</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>主齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1499,32 +1390,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-06 13:59:23</t>
+          <t>2026-10-14 16:20:44</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C01390021</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1534,67 +1430,77 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-27 13:59:36</t>
+          <t>2026-10-15 03:26:56</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01176034</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>二级大齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-14 18:15:12</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1604,50 +1510,10 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CC092679</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1664,7 +1530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1728,25 +1594,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>C01196422</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>高速齿轮轴组件#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>加工中心2</t>
+          <t>三坐标检测</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1756,19 +1622,19 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-13 15:55:41</t>
+          <t>2026-10-14 20:01:48</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>CC090193</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1796,19 +1662,19 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-11 01:37:19</t>
+          <t>2026-10-14 21:10:40</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1826,7 +1692,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1836,12 +1702,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-10 15:16:19</t>
+          <t>2026-10-14 18:27:31</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1853,25 +1719,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1881,42 +1747,37 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-13 10:55:27</t>
+          <t>2026-10-14 13:56:11</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>退磁</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300491</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1926,37 +1787,42 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-29 09:19:29</t>
+          <t>2026-10-14 13:59:03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196390</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1966,7 +1832,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 03:56:15</t>
+          <t>2026-10-13 10:55:27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1976,45 +1842,85 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>C01196395</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>齿轮轴</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-14 19:46:16</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>C01300253</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>摇臂钻2</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-10-13 18:17:38</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-14 19:43:21</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-15 09:33
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -608,12 +608,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C05000014</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>法兰</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -622,36 +622,41 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-13 13:04:07</t>
+          <t>2026-10-09 17:18:09</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-11-05 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C05000014</t>
+          <t>C01300541</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>法兰</t>
+          <t>Z326M6齿圈</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -660,46 +665,46 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-09 17:18:09</t>
+          <t>2026-10-10 16:02:04</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-11-05 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>CC090887</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -707,7 +712,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -717,40 +722,40 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
+          <t>2026-10-12 13:59:57</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196296</t>
+          <t>C01166011</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>消隙直齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -760,35 +765,40 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-13 13:39:35</t>
+          <t>2026-10-12 10:59:11</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CC090887</t>
+          <t>C01176035</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>二级消隙齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -798,40 +808,40 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:57</t>
+          <t>2026-10-12 11:12:30</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -841,22 +851,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:28</t>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -865,11 +880,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -879,183 +894,16 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-11-20 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>C01176035</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>二级消隙齿轮</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-12 11:12:30</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
         <v>1</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1069,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1287,25 +1135,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300491</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1315,24 +1163,24 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-14 18:05:38</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01196432</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>一二级高速轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1340,39 +1188,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-14 16:11:57</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196390</t>
+          <t>C01196434</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>三四级高速轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1380,39 +1223,34 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 16:20:44</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-14 16:18:01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01390021</t>
+          <t>C14006237</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1420,7 +1258,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1430,37 +1268,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-15 03:26:56</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-12 13:02:07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01176034</t>
+          <t>C01196425</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>二级大齿轮</t>
+          <t>高速齿轮轴27</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1470,50 +1303,510 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-14 18:15:12</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 08:36:29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>C14006261</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>推力环27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>锻造</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-15 08:37:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C01310054</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>厚齿圈</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>平面磨</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-07-27 13:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C01300491</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>主动同步齿轮</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-14 18:05:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C01310060</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>立磨</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-10-14 23:38:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C07000124</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>立磨</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-10-12 23:10:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C01000038</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>齿轮一</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-10-13 13:04:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C01196296</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-10-13 13:39:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C01300223</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>大齿轮组件</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>动平衡</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:54:55</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01196390</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>齿轮轴</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-14 16:20:44</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>C01390021</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>齿轮</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-10-15 03:26:56</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CC090888</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>齿轮（右）</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-10-12 13:59:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C01176034</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>二级大齿轮</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-10-14 18:15:12</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>CC092679</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D24" t="n">
         <v>3</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>加工中心</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>2026-06-03 14:50:03</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1608,7 +1901,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1622,12 +1915,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-14 20:01:48</t>
+          <t>2026-10-15 08:52:37</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-16 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,25 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300202</t>
+          <t>C01196422</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>高速齿轮轴组件#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,32 +507,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-11 12:55:33</t>
+          <t>2026-10-15 13:03:50</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01196210</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮轴组件</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -540,7 +540,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>检测</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -550,12 +550,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-14 10:26:31</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -565,17 +560,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01310018</t>
+          <t>C14006237</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -583,7 +578,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -593,27 +588,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17:49</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-12 13:02:07</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C05000014</t>
+          <t>C01310018</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>法兰</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -622,30 +612,30 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-09 17:18:09</t>
+          <t>2026-09-08 03:17:49</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-11-05 00:00:00</t>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -694,25 +684,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CC090887</t>
+          <t>C01196296</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -722,32 +712,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:57</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-13 13:39:35</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>C01196390</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -755,7 +740,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -765,12 +750,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
+          <t>2026-10-14 16:20:44</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -780,12 +765,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01176035</t>
+          <t>C01166011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>二级消隙齿轮</t>
+          <t>消隙直齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -808,7 +793,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 11:12:30</t>
+          <t>2026-10-12 10:59:11</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -823,12 +808,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01176035</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>二级消隙齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -837,11 +822,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -851,59 +836,140 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-15 15:47:08</t>
+          <t>2026-10-12 11:12:30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-01 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>XY06109</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>初级行星轮</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>滚齿2</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>2024-02-22 18:59:10</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>2026-11-20 00:00:00</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="I12" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -917,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1135,12 +1201,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196432</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>一二级高速轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1149,33 +1215,33 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-14 16:11:57</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196432</t>
+          <t>C01196434</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>一二级高速轴</t>
+          <t>三四级高速轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1198,24 +1264,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-14 16:11:57</t>
+          <t>2026-10-14 16:18:01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196434</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>三四级高速轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1223,29 +1289,34 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 16:18:01</t>
+          <t>2026-10-14 13:10:12</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C14006237</t>
+          <t>C01196425</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>高速齿轮轴27</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1254,33 +1325,33 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 13:02:07</t>
+          <t>2026-10-15 08:36:29</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01196425</t>
+          <t>C14006261</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>高速齿轮轴27</t>
+          <t>推力环27</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1289,7 +1360,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1303,19 +1374,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:36:29</t>
+          <t>2026-10-15 08:37:29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C14006261</t>
+          <t>C01310053</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>推力环27</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1324,21 +1395,21 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-15 08:37:29</t>
+          <t>2026-10-15 22:56:00</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1444,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-27 13:59:36</t>
+          <t>2026-10-15 23:45:54</t>
         </is>
       </c>
     </row>
@@ -1418,13 +1489,18 @@
           <t>C01310060</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>薄齿圈</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>子件</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1438,14 +1514,19 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-14 23:38:51</t>
+          <t>2026-10-15 15:34:46</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01310061</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1454,7 +1535,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1468,32 +1549,32 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-15 15:35:04</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C07000124</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1503,19 +1584,19 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-13 13:04:07</t>
+          <t>2026-10-12 23:10:08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01196296</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1524,11 +1605,11 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1538,24 +1619,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-13 13:39:35</t>
+          <t>2026-10-13 17:54:55</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01390021</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1563,7 +1649,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1573,24 +1659,24 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-10-15 03:26:56</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C01196390</t>
+          <t>C01390022</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1603,7 +1689,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1613,7 +1699,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-14 16:20:44</t>
+          <t>2026-10-15 16:06:59</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1625,12 +1711,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C01390021</t>
+          <t>C01390023</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>墨胶齿轮</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1653,7 +1739,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-15 03:26:56</t>
+          <t>2026-10-15 23:10:04</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1665,17 +1751,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01176033</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>一级大齿轮</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1683,7 +1769,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1693,7 +1779,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-10-12 13:59:28</t>
+          <t>2026-10-15 18:10:42</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1740,17 +1831,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>XY06110</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>输出行星轮</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1758,7 +1849,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>超精磨</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1768,45 +1859,10 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>CC092679</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
           <t>2026-06-03 14:50:03</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1823,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1887,25 +1943,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196422</t>
+          <t>C01300549</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>高速齿轮轴组件#</t>
+          <t>齿环#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>三坐标检测</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1915,17 +1971,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-15 08:52:37</t>
+          <t>2026-10-15 13:12:57</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2212,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2175,7 +2226,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 19:46:16</t>
+          <t>2026-10-15 15:03:06</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2187,38 +2238,83 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>C01196090</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-15 16:00:37</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>C01300253</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>19</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>摇臂钻2</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-10-14 19:43:21</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:08:00</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-17 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,25 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196422</t>
+          <t>C01310060</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>高速齿轮轴组件#</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,27 +507,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-15 13:03:50</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-22 00:00:00</t>
+          <t>2026-10-15 15:34:46</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01310061</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -536,11 +531,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -550,31 +545,31 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-15 15:35:04</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C14006237</t>
+          <t>C01300541</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>Z326M6齿圈</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -588,27 +583,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 13:02:07</t>
+          <t>2026-10-10 16:02:04</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01310018</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -616,7 +616,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,12 +626,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17:49</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-16 11:09:36</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -641,25 +636,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>C01166011</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>消隙直齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -669,40 +664,40 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
+          <t>2026-10-12 10:59:11</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196296</t>
+          <t>C01176033</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>一级大齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -712,27 +707,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 13:39:35</t>
+          <t>2026-10-15 18:10:42</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196390</t>
+          <t>C01176035</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>二级消隙齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -740,7 +740,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -750,12 +750,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 16:20:44</t>
+          <t>2026-10-12 11:12:30</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -765,12 +765,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -779,11 +779,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -793,27 +793,27 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
+          <t>2026-09-15 15:47:08</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-01 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01176035</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>二级消隙齿轮</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -822,11 +822,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -836,36 +836,36 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 11:12:30</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-11-20 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01300253</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -879,97 +879,11 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
+          <t>2026-10-16 17:56:46</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -983,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1201,35 +1115,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196432</t>
+          <t>C01196422</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>一二级高速轴</t>
+          <t>高速齿轮轴组件#</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-14 16:11:57</t>
+          <t>2026-10-15 13:03:50</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1230,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196425</t>
+          <t>C01310053</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>高速齿轮轴27</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1325,33 +1244,33 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-15 08:36:29</t>
+          <t>2026-10-15 22:56:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C14006261</t>
+          <t>C01310054</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>推力环27</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1360,46 +1279,46 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-15 08:37:29</t>
+          <t>2026-10-15 23:45:54</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01310053</t>
+          <t>C01310018</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1409,19 +1328,24 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-15 22:56:00</t>
+          <t>2026-09-08 03:17:49</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C14006096</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1430,11 +1354,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1444,19 +1368,19 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-15 23:45:54</t>
+          <t>2026-10-17 07:53:17</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300491</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1465,11 +1389,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1479,32 +1403,37 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-14 18:05:38</t>
+          <t>2026-10-13 17:54:55</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01310060</t>
+          <t>C01196390</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1514,24 +1443,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-15 15:34:46</t>
+          <t>2026-10-14 16:20:44</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01310061</t>
+          <t>C01390021</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1539,7 +1473,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1549,32 +1483,37 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-15 15:35:04</t>
+          <t>2026-10-15 03:26:56</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01390022</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1584,24 +1523,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-15 16:06:59</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01390023</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>墨胶齿轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1609,7 +1553,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1619,29 +1563,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-10-15 23:10:04</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01390021</t>
+          <t>C01176034</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>二级大齿轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1649,47 +1593,47 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-15 03:26:56</t>
+          <t>2026-10-14 18:15:12</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C01390022</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1699,170 +1643,10 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-15 16:06:59</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>C01390023</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>墨胶齿轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-10-15 23:10:04</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>C01176033</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>一级大齿轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>线切割</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-10-15 18:10:42</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>C01176034</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>二级大齿轮</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>线切割</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:15:12</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>CC092679</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1879,7 +1663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1983,25 +1767,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC090193</t>
+          <t>C01300565</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>输入转子组#</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>三坐标检测</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2011,19 +1795,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-14 21:10:40</t>
+          <t>2026-10-16 10:58:26</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>CC090193</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2037,38 +1826,33 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:10:40</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:27:31</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2082,7 +1866,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2096,12 +1880,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-14 13:56:11</t>
+          <t>2026-10-14 18:27:31</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>退磁</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
@@ -2171,7 +1960,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2181,7 +1970,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 10:55:27</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2198,25 +1987,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196395</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2226,12 +2015,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-15 15:03:06</t>
+          <t>2026-10-16 12:49:17</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
     </row>
@@ -2311,10 +2105,50 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-15 09:08:00</t>
+          <t>2026-10-16 18:50:43</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C01300254</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>齿轮（右）</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-16 18:50:39</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-18 08:53
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,12 +479,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01310060</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,11 +493,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,35 +507,35 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:34:46</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01310061</t>
+          <t>CC090193</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -545,35 +545,35 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-15 15:35:04</t>
+          <t>2026-10-17 08:53:45</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>C01310053</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -583,12 +583,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-15 22:56:00</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -598,12 +593,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01310054</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -612,11 +607,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,35 +621,35 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-16 11:09:36</t>
+          <t>2026-10-15 23:45:54</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01166011</t>
+          <t>C07000095</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>消隙直齿轮</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>打标</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -664,12 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-12 10:59:11</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-17 10:44:40</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -679,25 +669,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01176033</t>
+          <t>C01310060</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>一级大齿轮</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -707,40 +697,35 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-15 18:10:42</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 15:34:46</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01176035</t>
+          <t>C01310061</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>二级消隙齿轮</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -750,32 +735,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-12 11:12:30</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-17 12:39:56</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C07000124</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -783,7 +763,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -793,40 +773,35 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
+          <t>2026-10-12 23:10:08</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01300541</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>Z326M6齿圈</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -836,54 +811,340 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-10 16:02:04</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-11-20 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>C01300224</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-15 19:30:58</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C01300555</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:09:36</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C01176033</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>一级大齿轮</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:10:42</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C01196090</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:53:41</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-11-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>C01300253</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>6</v>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D18" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-16 17:56:46</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>7</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-17 18:11:09</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +1158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1075,17 +1336,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01310070</t>
+          <t>C01300549</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>外套</t>
+          <t>齿环#</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -1093,7 +1354,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1103,24 +1364,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-13 20:25:16</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-17 16:01:52</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196422</t>
+          <t>C01310070</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>高速齿轮轴组件#</t>
+          <t>外套</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1133,7 +1389,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1143,29 +1399,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-15 13:03:50</t>
+          <t>2026-10-13 20:25:16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>无断点</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196434</t>
+          <t>C01300565</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>三四级高速轴</t>
+          <t>输入转子组#</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1173,29 +1429,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-14 16:18:01</t>
+          <t>2026-10-17 10:18:55</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01300401</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1204,11 +1465,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1218,29 +1479,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 13:10:12</t>
+          <t>2026-10-16 17:48:45</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310053</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1248,7 +1509,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1258,32 +1519,37 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-15 22:56:00</t>
+          <t>2026-10-14 13:10:12</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C01300571</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>6X-205高速大轮#</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>渗碳淬火</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1293,32 +1559,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-15 23:45:54</t>
+          <t>2026-10-16 09:49:42</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01310018</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1328,37 +1594,37 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17:49</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>无断点</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C14006096</t>
+          <t>C01196395</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1368,24 +1634,24 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-17 07:53:17</t>
+          <t>2026-10-17 09:23:07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01300081</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1393,7 +1659,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1403,29 +1669,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-10-16 22:21:01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01196390</t>
+          <t>BXZ00003</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>行走减速机</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1433,7 +1699,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1443,37 +1709,37 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-14 16:20:44</t>
+          <t>2026-10-17 10:26:08</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>无断点</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01390021</t>
+          <t>C14006096</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1483,37 +1749,32 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-15 03:26:56</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-17 11:16:47</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01390022</t>
+          <t>C14006221</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>轴套2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>精车</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1523,29 +1784,24 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-15 16:06:59</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-16 23:09:27</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01390023</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>墨胶齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1553,7 +1809,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1563,29 +1819,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-15 23:10:04</t>
+          <t>2026-10-13 17:54:55</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01176034</t>
+          <t>C01390023</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>二级大齿轮</t>
+          <t>墨胶齿轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1593,60 +1849,100 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-14 18:15:12</t>
+          <t>2026-10-15 23:10:04</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>C01176034</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>二级大齿轮</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-14 18:15:12</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>CC092679</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D20" t="n">
         <v>3</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>加工中心</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>2026-06-03 14:50:03</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>
@@ -1663,7 +1959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1727,25 +2023,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300549</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿环#</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1755,37 +2051,42 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-15 13:12:57</t>
+          <t>2026-10-14 18:27:31</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300565</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>输入转子组#</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>三坐标检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1795,24 +2096,19 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-16 10:58:26</t>
+          <t>2026-10-14 13:56:11</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-10-22 00:00:00</t>
+          <t>退磁</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090193</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1826,11 +2122,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1840,69 +2136,74 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-14 21:10:40</t>
+          <t>2026-10-14 13:59:03</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>C01196179</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>高速齿轮组27</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-18 04:27:21</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:27:31</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1911,101 +2212,101 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-16 12:49:17</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-14 13:59:03</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-10-17 11:31:39</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:17:13</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>C01196411</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>输入齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2015,7 +2316,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-16 12:49:17</t>
+          <t>2026-10-18 06:37:20</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2025,32 +2326,32 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196090</t>
+          <t>C01300253</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2060,7 +2361,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-15 16:00:37</t>
+          <t>2026-10-17 09:42:15</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2070,19 +2371,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300253</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2091,7 +2392,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2105,50 +2406,10 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-16 18:50:43</t>
+          <t>2026-10-17 09:42:01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>C01300254</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>齿轮（右）</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>6</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>摇臂钻2</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-16 18:50:39</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-19 08:54
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,25 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300565</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>输入转子组#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,7 +507,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-17 10:18:55</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -517,17 +522,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC090193</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -535,7 +540,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -545,7 +550,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-17 08:53:45</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -555,17 +560,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01310053</t>
+          <t>CC090193</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -573,7 +578,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -583,22 +588,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-15 22:56:00</t>
+          <t>2026-10-17 08:53:45</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C01310053</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -621,7 +626,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-15 23:45:54</t>
+          <t>2026-10-15 22:56:00</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -631,12 +636,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C07000095</t>
+          <t>C01310054</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -649,7 +654,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>打标</t>
+          <t>平面磨</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,22 +664,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-17 10:44:40</t>
+          <t>2026-10-15 23:45:54</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01310060</t>
+          <t>C07000095</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -683,11 +688,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>打标</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -697,7 +702,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-15 15:34:46</t>
+          <t>2026-10-17 10:44:40</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -707,12 +712,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01310061</t>
+          <t>C01310060</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>薄齿圈</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -735,7 +740,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-17 12:39:56</t>
+          <t>2026-10-15 15:34:46</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -745,12 +750,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01310061</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -773,7 +778,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-17 12:39:56</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -783,17 +788,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>C07000124</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>轮毂</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -801,7 +806,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -811,12 +816,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-12 23:10:08</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -826,25 +826,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300224</t>
+          <t>C01196395</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -854,31 +854,31 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-15 19:30:58</t>
+          <t>2026-10-17 09:23:07</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01300541</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>Z326M6齿圈</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -892,35 +892,40 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-16 11:09:36</t>
+          <t>2026-10-10 16:02:04</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01176033</t>
+          <t>C14006096</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>一级大齿轮</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -930,40 +935,35 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-15 18:10:42</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-17 11:16:47</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01196090</t>
+          <t>C14006221</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>轴套2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -973,40 +973,35 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-17 08:53:41</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-16 23:09:27</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01300224</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1016,40 +1011,35 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
+          <t>2026-10-15 19:30:58</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1059,27 +1049,22 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
+          <t>2026-10-16 11:09:36</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XY06110</t>
+          <t>C01176033</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>输出行星轮</t>
+          <t>一级大齿轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1088,11 +1073,11 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>超精磨</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1102,49 +1087,221 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2025-04-17 10:57:01</t>
+          <t>2026-10-15 18:10:42</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>C01196090</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:53:41</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:47:08</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-11-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>C01300253</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>齿轮（左）</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>油气</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D22" t="n">
         <v>14</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>2026-10-17 18:11:09</t>
         </is>
       </c>
-      <c r="I18" t="n">
-        <v>14</v>
+      <c r="I22" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1158,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1411,12 +1568,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300565</t>
+          <t>C01300401</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>输入转子组#</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1425,11 +1582,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1439,24 +1596,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-17 10:18:55</t>
+          <t>2026-10-16 17:48:45</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-22 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300401</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1465,11 +1622,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1479,37 +1636,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-16 17:48:45</t>
+          <t>2026-10-14 13:10:12</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01300571</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>6X-205高速大轮#</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>渗碳淬火</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1519,37 +1676,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-14 13:10:12</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-16 09:49:42</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300571</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6X-205高速大轮#</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>渗碳淬火</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1559,32 +1711,37 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-16 09:49:42</t>
+          <t>2026-10-16 15:17:13</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>C01300081</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1594,37 +1751,37 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-16 15:17:13</t>
+          <t>2026-10-16 22:21:01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01196395</t>
+          <t>BXZ00003</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>行走减速机</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1634,24 +1791,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-17 09:23:07</t>
+          <t>2026-10-17 10:26:08</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300081</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1659,7 +1821,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1669,29 +1831,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-16 22:21:01</t>
+          <t>2026-10-13 17:54:55</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BXZ00003</t>
+          <t>C01390023</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>行走减速机</t>
+          <t>墨胶齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1699,7 +1861,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1709,72 +1871,77 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-17 10:26:08</t>
+          <t>2026-10-15 23:10:04</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C14006096</t>
+          <t>C01176034</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>二级大齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-17 11:16:47</t>
+          <t>2026-10-14 18:15:12</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C14006221</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>轴套2</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>精车</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1784,165 +1951,10 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-16 23:09:27</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>C01300223</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>大齿轮组件</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>动平衡</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-10-13 17:54:55</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>C01390023</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>墨胶齿轮</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-10-15 23:10:04</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>C01176034</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>二级大齿轮</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>线切割</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:15:12</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CC092679</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
           <t>2026-06-03 14:50:03</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>2026-10-15 00:00:00</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-20 09:31
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,12 +479,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300565</t>
+          <t>C01300545</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>输入转子组#</t>
+          <t>内套I#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,26 +493,26 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-17 10:18:55</t>
+          <t>2026-10-12 10:46:14</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-22 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -522,17 +522,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300546</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>内套II#</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -540,17 +540,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-12 10:46:15</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -560,17 +565,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090193</t>
+          <t>C01300547</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>内套I</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -578,17 +583,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-17 08:53:45</t>
+          <t>2026-10-12 10:46:14</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -598,25 +608,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01310053</t>
+          <t>C01300253</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,60 +636,65 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-15 22:56:00</t>
+          <t>2026-10-19 18:29:16</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:30:37</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>平面磨</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-15 23:45:54</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C07000095</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -692,7 +707,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>打标</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -702,35 +717,35 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-17 10:44:40</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01310060</t>
+          <t>C01300401</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>薄齿圈</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -740,35 +755,40 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-15 15:34:46</t>
+          <t>2026-10-16 17:48:45</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310061</t>
+          <t>C01196395</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -778,35 +798,35 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-17 12:39:56</t>
+          <t>2026-10-17 09:23:07</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C07000124</t>
+          <t>C01300081</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>轮毂</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -816,31 +836,36 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-12 23:10:08</t>
+          <t>2026-10-16 22:21:01</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196395</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -854,35 +879,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-17 09:23:07</t>
+          <t>2026-10-19 13:28:03</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300541</t>
+          <t>C14006096</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Z326M6齿圈</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -892,27 +922,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-10 16:02:04</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-17 11:16:47</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C14006096</t>
+          <t>C14006221</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>轴套2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -921,11 +946,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>精车</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -935,35 +960,35 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-17 11:16:47</t>
+          <t>2026-10-16 23:09:27</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C14006221</t>
+          <t>C01390023</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>轴套2</t>
+          <t>墨胶齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>精车</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -973,31 +998,36 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-16 23:09:27</t>
+          <t>2026-10-15 23:10:04</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01300224</t>
+          <t>C01176034</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>二级大齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1006,32 +1036,37 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-15 19:30:58</t>
+          <t>2026-10-14 18:15:12</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1049,22 +1084,27 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-16 11:09:36</t>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01176033</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>一级大齿轮</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1073,11 +1113,11 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1087,27 +1127,27 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-15 18:10:42</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-11-20 00:00:00</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01196090</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1116,11 +1156,11 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1130,178 +1170,11 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-17 08:53:41</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
         <v>3</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-09-15 15:47:08</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-10-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>C01300253</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>14</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-10-17 18:11:09</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1315,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1373,17 +1246,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300545</t>
+          <t>C01300549</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>内套I#</t>
+          <t>齿环#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1391,34 +1264,29 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-17 16:01:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300546</t>
+          <t>C01310070</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>内套II#</t>
+          <t>外套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1431,17 +1299,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:15</t>
+          <t>2026-10-13 20:25:16</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1453,65 +1321,65 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300547</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>内套I</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300549</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿环#</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1521,32 +1389,37 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-17 16:01:52</t>
+          <t>2026-10-14 13:10:12</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01310070</t>
+          <t>C01300571</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>外套</t>
+          <t>6X-205高速大轮#</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>渗碳淬火</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1556,24 +1429,24 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-13 20:25:16</t>
+          <t>2026-10-19 08:38:51</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300401</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1582,11 +1455,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1596,29 +1469,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-16 17:48:45</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>BXZ00003</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>行走减速机</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1626,7 +1499,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1636,37 +1509,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-14 13:10:12</t>
+          <t>2026-10-17 10:26:08</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-12-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300571</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6X-205高速大轮#</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>渗碳淬火</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1676,287 +1549,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-16 09:49:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>C01300322</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>主动同步齿轮</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:17:13</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>C01300081</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>齿轮</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>线切割</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-16 22:21:01</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-08 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BXZ00003</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>行走减速机</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>齿轮箱</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>装配</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-17 10:26:08</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-20 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C01300223</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>大齿轮组件</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>动平衡</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
           <t>2026-10-13 17:54:55</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>C01390023</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>墨胶齿轮</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-10-15 23:10:04</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>C01176034</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>二级大齿轮</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>线切割</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:15:12</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CC092679</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>齿轮（左）</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2035,92 +1633,87 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>C01196396</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>轴齿轮#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>齿检仪检测</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:52:17</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:27:31</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-10-17 09:42:01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-10-14 13:56:11</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>退磁</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2148,7 +1741,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-14 13:59:03</t>
+          <t>2026-10-14 18:27:31</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2165,25 +1758,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196179</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>高速齿轮组27</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2193,29 +1786,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-18 04:27:21</t>
+          <t>2026-10-14 13:56:11</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>退磁</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2224,11 +1812,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2238,34 +1826,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-16 12:49:17</t>
+          <t>2026-10-14 13:59:03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01196179</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>高速齿轮组27</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -2283,7 +1871,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-17 11:31:39</t>
+          <t>2026-10-18 04:27:21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2293,32 +1881,32 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196411</t>
+          <t>C01196385</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>高速齿轮组41</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2328,42 +1916,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-18 06:37:20</t>
+          <t>2026-10-20 05:57:57</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300253</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2373,57 +1956,147 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-17 09:42:15</t>
+          <t>2026-10-19 15:32:09</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-17 09:42:01</t>
+          <t>2026-10-19 14:08:30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C01196393</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>涡轮轴</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-17 11:31:39</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C01196411</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-18 06:37:20</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-21 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -608,7 +608,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300253</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -622,11 +622,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -636,40 +636,40 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-19 18:29:16</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-19 18:30:37</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -689,25 +689,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>CC090685</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -717,27 +717,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-20 15:26:27</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300401</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -745,7 +750,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -755,12 +760,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-16 17:48:45</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-20 15:24:24</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -770,25 +770,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196395</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -798,35 +798,40 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-17 09:23:07</t>
+          <t>2026-10-20 15:23:32</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300081</t>
+          <t>C01300401</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -836,36 +841,36 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-16 22:21:01</t>
+          <t>2026-10-16 17:48:45</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -879,40 +884,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-19 13:28:03</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C14006096</t>
+          <t>C01300081</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -922,35 +927,40 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-17 11:16:47</t>
+          <t>2026-10-16 22:21:01</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C14006221</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>轴套2</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>精车</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -960,35 +970,40 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-16 23:09:27</t>
+          <t>2026-10-19 13:28:03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01390023</t>
+          <t>C14006096</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>墨胶齿轮</t>
+          <t>推力盘</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -998,75 +1013,65 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-15 23:10:04</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-17 11:16:47</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01176034</t>
+          <t>C14006221</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>二级大齿轮</t>
+          <t>轴套2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>精车</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-14 18:15:12</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-16 23:09:27</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1074,7 +1079,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1084,40 +1089,40 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-14 16:14:17</t>
+          <t>2026-10-13 17:54:55</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>无断点</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1127,53 +1132,172 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-11-20 00:00:00</t>
+          <t>2026-10-20 23:47:25</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>C01390023</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>墨胶齿轮</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-15 23:10:04</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>无断点</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>XY06110</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>输出行星轮</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D21" t="n">
         <v>3</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>超精磨</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>2025-04-17 10:57:01</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="I21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1188,7 +1312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1264,7 +1388,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1274,7 +1398,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-17 16:01:52</t>
+          <t>2026-10-20 21:10:54</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1445,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC092679</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1335,7 +1459,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1349,37 +1473,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-20 14:49:43</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1389,64 +1508,59 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-14 13:10:12</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 18:05:04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300571</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6X-205高速大轮#</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>渗碳淬火</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-19 08:38:51</t>
+          <t>2026-10-17 09:20:27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1455,11 +1569,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1469,37 +1583,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-16 15:17:13</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-13 15:21:27</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BXZ00003</t>
+          <t>C01300571</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>行走减速机</t>
+          <t>6X-205高速大轮#</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>渗碳淬火</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1509,52 +1618,127 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-17 10:26:08</t>
+          <t>2026-10-19 08:38:51</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-12-20 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01310054</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>厚齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>平面磨</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-07-27 13:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BXZ00003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>行走减速机</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>齿轮箱</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>2</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>动平衡</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-10-13 17:54:55</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>装配</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-10-17 10:26:08</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-12-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C01196411</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-20 18:06:59</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1673,25 +1857,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C07000134</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>外圆磨2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1701,7 +1885,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-17 09:42:01</t>
+          <t>2026-10-20 19:18:57</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1713,12 +1897,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1731,39 +1915,39 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:33:46</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-10-14 18:27:31</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1772,83 +1956,83 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:33:49</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-14 13:56:11</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>退磁</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>C01196179</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>高速齿轮组27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-18 04:27:21</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-14 13:59:03</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196179</t>
+          <t>C01196385</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高速齿轮组27</t>
+          <t>高速齿轮组41</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1871,7 +2055,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-18 04:27:21</t>
+          <t>2026-10-21 01:52:27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1881,24 +2065,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196385</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高速齿轮组41</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1906,7 +2090,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1916,24 +2100,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-20 05:57:57</t>
+          <t>2026-10-19 15:32:09</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1942,7 +2131,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1951,34 +2140,29 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-19 15:32:09</t>
+          <t>2026-10-19 14:08:30</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1987,38 +2171,43 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-19 14:08:30</t>
+          <t>2026-10-17 11:31:39</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2041,7 +2230,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-17 11:31:39</t>
+          <t>2026-10-20 16:47:26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2052,51 +2241,6 @@
       <c r="I11" t="inlineStr">
         <is>
           <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>C01196411</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>输入齿轮轴</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-18 06:37:20</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-22 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -608,25 +608,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CC092679</t>
+          <t>C01300549</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>齿环#</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -636,40 +636,35 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-20 21:10:54</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -679,35 +674,35 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-20 18:05:04</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CC090685</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -717,7 +712,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-20 15:26:27</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -726,23 +721,23 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -750,7 +745,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -760,7 +755,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-20 15:24:24</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -770,7 +765,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>CC091366</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -784,7 +779,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -798,40 +793,35 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-20 15:23:32</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-20 15:24:24</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300401</t>
+          <t>CC091386</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -841,27 +831,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-16 17:48:45</t>
+          <t>2026-10-20 15:23:32</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>C01300401</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -870,11 +860,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -884,40 +874,40 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-16 15:17:13</t>
+          <t>2026-10-16 17:48:45</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300081</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -927,27 +917,27 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-16 22:21:01</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>C01300081</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -956,11 +946,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -970,7 +960,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-19 13:28:03</t>
+          <t>2026-10-16 22:21:01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -979,31 +969,31 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C14006096</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>推力盘</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1013,35 +1003,40 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-17 11:16:47</t>
+          <t>2026-10-19 13:28:03</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C14006221</t>
+          <t>XZ00338</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>轴套2</t>
+          <t>行走齿轮箱</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>精车</t>
+          <t>喷漆</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1051,35 +1046,40 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-16 23:09:27</t>
+          <t>2026-10-21 09:16:50</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-28 00:00:00</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>XZ00090</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>SMAT TR25 B轴齿轮箱</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>喷漆</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-10-21 09:12:57</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1104,17 +1104,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>BXZ00003</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>行走减速机</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1132,7 +1132,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-20 23:47:25</t>
+          <t>2026-10-17 10:26:08</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-12-20 00:00:00</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1142,17 +1147,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01390023</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>墨胶齿轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1160,7 +1165,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1170,32 +1175,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-15 23:10:04</t>
+          <t>2026-10-13 17:54:55</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1203,7 +1208,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1213,27 +1218,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>无断点</t>
+          <t>2026-10-20 23:47:25</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01196411</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>输入齿轮轴</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1242,11 +1242,11 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1256,48 +1256,134 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-20 18:06:59</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>无断点</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>XY06110</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>输出行星轮</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D23" t="n">
         <v>3</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>超精磨</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>2025-04-17 10:57:01</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="I23" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1370,17 +1456,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300549</t>
+          <t>C01310070</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿环#</t>
+          <t>外套</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1388,7 +1474,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1398,32 +1484,37 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-20 21:10:54</t>
+          <t>2026-10-13 20:25:16</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01310070</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>外套</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1433,19 +1524,14 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-13 20:25:16</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-21 15:26:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1455,15 +1541,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1473,42 +1559,52 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-20 14:49:43</t>
+          <t>2026-10-21 15:54:16</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-20 18:05:04</t>
+          <t>2026-10-17 09:20:27</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1529,26 +1625,21 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-17 09:20:27</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-21 15:55:01</t>
         </is>
       </c>
     </row>
@@ -1630,17 +1721,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310054</t>
+          <t>C01300339</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>厚齿圈</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1648,7 +1739,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>平面磨</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1658,32 +1749,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-27 13:59:36</t>
+          <t>2026-10-21 16:44:24</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BXZ00003</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>行走减速机</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1693,33 +1784,28 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-17 10:26:08</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-12-20 00:00:00</t>
+          <t>2026-10-21 18:16:11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196411</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1733,12 +1819,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-20 18:06:59</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
+          <t>2026-10-21 14:00:51</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1897,35 +1978,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01196179</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>高速齿轮组27</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-20 09:33:46</t>
+          <t>2026-10-18 04:27:21</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1935,72 +2016,77 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01196385</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>高速齿轮组41</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-20 09:33:49</t>
+          <t>2026-10-21 01:52:27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196179</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>高速齿轮组27</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2010,34 +2096,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-18 04:27:21</t>
+          <t>2026-10-21 14:17:32</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196385</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高速齿轮组41</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -2055,7 +2141,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-21 01:52:27</t>
+          <t>2026-10-17 11:31:39</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2065,19 +2151,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2090,7 +2176,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2100,52 +2186,52 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-19 15:32:09</t>
+          <t>2026-10-20 16:47:26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-19 14:08:30</t>
+          <t>2026-10-22 07:53:10</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2153,94 +2239,9 @@
           <t>磁粉探伤</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>C01196393</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>涡轮轴</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>外圆磨</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:31:39</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>C01196394</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>输入轴</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>外圆磨</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-20 16:47:26</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-23 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -48,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,17 +480,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300545</t>
+          <t>C01196396</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>内套I#</t>
+          <t>轴齿轮#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -497,22 +498,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-22 13:55:54</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -522,12 +518,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300546</t>
+          <t>C01300545</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>内套II#</t>
+          <t>内套I#</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -550,7 +546,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:15</t>
+          <t>2026-10-12 10:46:14</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -565,12 +561,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300547</t>
+          <t>C01300546</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>内套I</t>
+          <t>内套II#</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -593,7 +589,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
+          <t>2026-10-12 10:46:15</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -608,17 +604,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300549</t>
+          <t>C01300547</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿环#</t>
+          <t>内套I</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -631,12 +627,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-20 21:10:54</t>
+          <t>2026-10-12 10:46:14</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -646,12 +647,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -660,11 +661,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -674,8 +675,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-20 18:05:04</t>
-        </is>
+          <t>2026-06-03 14:50:03</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>3</v>
@@ -684,25 +688,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CC092679</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -712,40 +716,35 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -755,22 +754,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-21 15:54:16</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CC091366</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -783,32 +787,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-20 15:24:24</t>
+          <t>2026-10-17 09:20:27</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CC091386</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -817,11 +826,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,27 +840,22 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-20 15:23:32</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-21 15:55:01</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300401</t>
+          <t>C01300322</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>主动同步齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -860,11 +864,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -874,36 +878,36 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-16 17:48:45</t>
+          <t>2026-10-16 15:17:13</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>C01300355</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>小齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -917,16 +921,14 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-16 15:17:13</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
-        </is>
+          <t>2026-10-19 13:28:03</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -975,12 +977,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -993,7 +995,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1003,12 +1005,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-19 13:28:03</t>
+          <t>2026-10-22 09:35:30</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1018,25 +1020,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XZ00338</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>行走齿轮箱</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>喷漆</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1046,40 +1048,35 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-21 09:16:50</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-28 00:00:00</t>
+          <t>2026-10-20 23:47:25</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XZ00090</t>
+          <t>C01300223</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SMAT TR25 B轴齿轮箱</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>喷漆</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1089,40 +1086,40 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-21 09:12:57</t>
+          <t>2026-10-13 17:54:55</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BXZ00003</t>
+          <t>C01196057</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>行走减速机</t>
+          <t>高速轴1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1132,40 +1129,35 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-17 10:26:08</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-12-20 00:00:00</t>
+          <t>2026-10-20 10:07:40</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01196411</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>输入齿轮轴</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1175,32 +1167,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
+          <t>2026-10-20 18:06:59</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1208,7 +1200,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1218,22 +1210,27 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-20 23:47:25</t>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C01196411</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1242,11 +1239,11 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1256,27 +1253,22 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-10-20 18:06:59</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1285,11 +1277,11 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1299,91 +1291,10 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>无断点</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1398,7 +1309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1456,25 +1367,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01310070</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>外套</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1484,12 +1395,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-13 20:25:16</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 18:05:04</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1416,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1524,32 +1430,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-21 15:26:55</t>
+          <t>2026-10-22 14:41:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1559,73 +1465,68 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-21 15:54:16</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-13 15:21:27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300571</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>6X-205高速大轮#</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>渗碳淬火</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-17 09:20:27</t>
+          <t>2026-10-19 08:38:51</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01196385</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>高速齿轮组41</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1639,19 +1540,24 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-21 15:55:01</t>
+          <t>2026-10-22 14:34:11</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01300339</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1664,7 +1570,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1674,32 +1580,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-21 16:44:24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300571</t>
+          <t>C01196179</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6X-205高速大轮#</t>
+          <t>高速齿轮组27</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>渗碳淬火</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1709,37 +1615,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-19 08:38:51</t>
+          <t>2026-10-22 14:34:04</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300339</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1749,19 +1655,19 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-21 16:44:24</t>
+          <t>2026-10-21 18:16:11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1770,7 +1676,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1784,19 +1690,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-21 18:16:11</t>
+          <t>2026-10-21 14:00:51</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>CC091566</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1809,17 +1715,87 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:22:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C01196025</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>低速小齿轮</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-21 14:00:51</t>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:00:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>XZ00291</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>行走齿轮箱（不含马达）</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>齿轮箱</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>装配</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:00:25</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1898,17 +1874,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196396</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>轴齿轮#</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1916,7 +1892,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1926,7 +1902,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-19 19:52:17</t>
+          <t>2026-10-22 19:38:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1978,12 +1954,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196179</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>高速齿轮组27</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1992,7 +1968,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2006,42 +1982,37 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-18 04:27:21</t>
+          <t>2026-10-23 02:40:50</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-10-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196385</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>高速齿轮组41</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>立磨</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2051,29 +2022,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-21 01:52:27</t>
+          <t>2026-10-22 23:42:34</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2082,43 +2048,43 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-17 11:31:39</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-21 14:17:32</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>退磁</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2127,7 +2093,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2141,7 +2107,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-17 11:31:39</t>
+          <t>2026-10-20 16:47:26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2158,25 +2124,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2186,7 +2152,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-20 16:47:26</t>
+          <t>2026-10-22 07:53:10</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2195,51 +2161,6 @@
         </is>
       </c>
       <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>C01310072</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>大齿圈</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-10-22 07:53:10</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
         <is>
           <t>2026-10-06 00:00:00</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-24 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -48,9 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -518,103 +517,98 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300545</t>
+          <t>CC092679</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>内套I#</t>
+          <t>齿轮（左）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
+          <t>2026-06-03 14:50:03</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300546</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>内套II#</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:15</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 18:05:04</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300547</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>内套I</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -622,22 +616,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-12 10:46:14</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -647,25 +636,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC092679</t>
+          <t>CC090194</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -675,38 +664,35 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>0</v>
+          <t>2026-10-23 16:34:49</t>
+        </is>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -716,17 +702,22 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-21 15:54:16</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -740,7 +731,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -754,7 +745,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-21 15:54:16</t>
+          <t>2026-10-21 15:55:01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -763,74 +754,74 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300339</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>动平衡</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-23 15:26:18</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>外圆磨</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-10-17 09:20:27</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300533</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -840,35 +831,40 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-21 15:55:01</t>
+          <t>2026-10-23 09:37:06</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300322</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>主动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -878,27 +874,27 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-16 15:17:13</t>
+          <t>2026-10-22 09:35:30</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300355</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>小齿轮</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -907,7 +903,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -921,25 +917,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-19 13:28:03</t>
-        </is>
-      </c>
-      <c r="H12" s="1" t="n">
-        <v>0</v>
+          <t>2026-10-21 18:16:11</t>
+        </is>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300081</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -952,7 +945,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -962,12 +955,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-16 22:21:01</t>
+          <t>2026-10-23 13:00:35</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-08 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -977,25 +970,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1005,27 +998,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-22 09:35:30</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2026-10-20 23:47:25</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01196025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>低速小齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1034,11 +1022,11 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1048,35 +1036,35 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-20 23:47:25</t>
+          <t>2026-10-22 19:00:07</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01300223</t>
+          <t>C01196057</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>高速轴1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1086,40 +1074,35 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-13 17:54:55</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 10:07:40</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01196057</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>高速轴1</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1129,22 +1112,27 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-20 10:07:40</t>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01196411</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>输入齿轮轴</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1153,11 +1141,11 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,27 +1155,22 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-20 18:06:59</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1196,11 +1179,11 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1210,91 +1193,10 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>无断点</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1309,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1367,12 +1269,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1381,11 +1283,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1395,32 +1297,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-20 18:05:04</t>
+          <t>2026-10-22 14:41:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1430,19 +1332,19 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-22 14:41:55</t>
+          <t>2026-10-13 15:21:27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1451,11 +1353,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1465,32 +1367,37 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-23 16:20:30</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300571</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6X-205高速大轮#</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>渗碳淬火</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1500,37 +1407,32 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-19 08:38:51</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196385</t>
+          <t>CC091566</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>高速齿轮组41</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1540,37 +1442,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-22 14:34:11</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-23 04:22:18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300339</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1580,24 +1477,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-21 16:44:24</t>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196179</t>
+          <t>CC090888</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高速齿轮组27</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1605,7 +1507,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1615,37 +1517,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-22 14:34:04</t>
+          <t>2026-10-23 19:38:15</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>XZ00291</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>行走齿轮箱（不含马达）</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1655,147 +1557,47 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-21 18:16:11</t>
+          <t>2026-10-22 15:00:25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-21 14:00:51</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CC091566</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>齿圈</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-23 04:22:18</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>C01196025</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>低速小齿轮</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>子件</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-22 19:00:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>XZ00291</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>行走齿轮箱（不含马达）</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>齿轮箱</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>装配</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-10-22 15:00:25</t>
+          <t>2026-10-23 16:36:38</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1888,7 +1690,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1902,7 +1704,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-22 19:38:00</t>
+          <t>2026-10-23 15:01:14</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1954,21 +1756,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1982,37 +1784,42 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-23 02:40:50</t>
+          <t>2026-10-17 11:31:39</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>立磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2022,7 +1829,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-22 23:42:34</t>
+          <t>2026-10-22 07:53:10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2030,137 +1837,7 @@
           <t>磁粉探伤</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>C01196393</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>涡轮轴</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>外圆磨</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-17 11:31:39</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>C01196394</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>输入轴</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>外圆磨</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-10-20 16:47:26</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>C01310072</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>大齿圈</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-10-22 07:53:10</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>2026-10-06 00:00:00</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-25 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,25 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196396</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>轴齿轮#</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,35 +507,35 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-22 13:55:54</t>
+          <t>2026-10-22 14:41:55</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC092679</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮（左）</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -545,40 +545,35 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-03 14:50:03</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>CC090194</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -588,35 +583,35 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-20 18:05:04</t>
+          <t>2026-10-23 16:34:49</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -626,22 +621,27 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-21 15:54:16</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC090194</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -650,11 +650,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -664,35 +664,40 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23 16:34:49</t>
+          <t>2026-10-21 15:55:01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -702,40 +707,40 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-21 15:54:16</t>
+          <t>2026-10-13 15:21:27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -745,27 +750,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-21 15:55:01</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-24 15:45:06</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300339</t>
+          <t>C01300388</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 15:26:18</t>
+          <t>2026-10-24 18:29:46</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -803,7 +803,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300533</t>
+          <t>C01300339</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -831,32 +831,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 09:37:06</t>
+          <t>2026-10-23 15:26:18</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01300533</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-22 09:35:30</t>
+          <t>2026-10-23 09:37:06</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -889,12 +889,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>CC092697</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -903,11 +903,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -917,22 +917,27 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-21 18:16:11</t>
+          <t>2026-10-22 09:35:30</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-11-01 00:00:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -941,7 +946,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -955,32 +960,27 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-21 18:16:11</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -988,7 +988,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -998,7 +998,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-20 23:47:25</t>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1008,25 +1013,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01196025</t>
+          <t>CC091566</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>低速小齿轮</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1036,22 +1041,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-22 19:00:07</t>
+          <t>2026-10-24 13:21:59</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01196057</t>
+          <t>C01300555</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>高速轴1</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1060,11 +1070,11 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1074,35 +1084,35 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-20 10:07:40</t>
+          <t>2026-10-20 23:47:25</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01216011</t>
+          <t>C01196057</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>中间级行星轮</t>
+          <t>高速轴1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1112,40 +1122,35 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>无断点</t>
+          <t>2026-10-20 10:07:40</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1155,48 +1160,134 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>无断点</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>XY06110</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>输出行星轮</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D21" t="n">
         <v>3</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>超精磨</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>2025-04-17 10:57:01</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="I21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1211,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1269,25 +1360,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>JC095136</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>一级行星轮</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>清理喷丸</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1297,28 +1388,33 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-22 14:41:55</t>
+          <t>2026-10-24 17:57:12</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01196254</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>低速齿轮轴46</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1332,7 +1428,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-24 19:56:51</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1510,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC091566</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1432,7 +1528,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1442,32 +1538,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23 04:22:18</t>
+          <t>2026-10-24 13:15:22</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C01196349</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1477,24 +1573,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-24 19:55:12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1503,11 +1594,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1517,37 +1608,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-23 19:38:15</t>
+          <t>2026-10-24 13:28:41</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>XZ00291</t>
+          <t>C01310074</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>行走齿轮箱（不含马达）</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1557,45 +1648,125 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-22 15:00:25</t>
+          <t>2026-10-25 07:17:52</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-11-04 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>CC090888</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>齿轮（右）</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:38:15</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>XZ00291</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>行走齿轮箱（不含马达）</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>齿轮箱</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>装配</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:00:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>C01000061</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>油泵齿轮</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>齿轮箱-高精</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>调质</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>委外-完工</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>2026-10-23 16:36:38</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>2026-12-15 00:00:00</t>
         </is>
@@ -1612,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1798,51 +1969,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>C01310072</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>大齿圈</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-22 07:53:10</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-26 08:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -1056,12 +1056,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01300555</t>
+          <t>C01196057</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>高速轴1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1070,11 +1070,11 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1084,35 +1084,35 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-20 23:47:25</t>
+          <t>2026-10-20 10:07:40</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C01196057</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>高速轴1</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1122,31 +1122,36 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-10-20 10:07:40</t>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1160,16 +1165,16 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
+          <t>2026-10-24 13:28:41</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1360,25 +1365,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JC095136</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>一级行星轮</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>清理喷丸</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1388,37 +1393,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-24 17:57:12</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-25 10:31:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01196254</t>
+          <t>JC095136</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>低速齿轮轴46</t>
+          <t>一级行星轮</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>风电项目（非远景）</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>清理喷丸</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1428,24 +1428,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-24 19:56:51</t>
+          <t>2026-10-24 17:57:12</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01196254</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>低速齿轮轴46</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -1453,7 +1458,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1463,33 +1468,28 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:30</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-24 19:56:51</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1503,24 +1503,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-23 16:20:30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1528,7 +1533,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1538,32 +1543,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-24 13:15:22</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1573,32 +1578,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-24 19:55:12</t>
+          <t>2026-10-24 13:15:22</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01310072</t>
+          <t>C01196349</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>大齿圈</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1608,12 +1613,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-24 13:28:41</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-25 16:52:31</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1966,6 +1966,51 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>2026-10-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C01196092</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>二级齿轮轴</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>加工中心3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-25 23:21:25</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-26 14:42
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -479,12 +479,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,11 +493,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,35 +507,35 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-22 14:41:55</t>
+          <t>2026-10-25 10:31:12</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -545,27 +545,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-22 14:41:55</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090194</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -573,7 +573,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -583,7 +583,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-23 16:34:49</t>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -593,25 +598,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,40 +626,35 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-21 15:54:16</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-24 15:45:06</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300388</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -664,40 +664,40 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-21 15:55:01</t>
+          <t>2026-10-24 18:29:46</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -707,40 +707,35 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-21 18:16:11</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -750,35 +745,40 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-24 15:45:06</t>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300388</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -788,32 +788,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-24 18:29:46</t>
+          <t>2026-10-24 13:28:41</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300339</t>
+          <t>C01310074</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -821,7 +821,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 15:26:18</t>
+          <t>2026-10-25 07:17:52</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-11-04 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -846,17 +846,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300533</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -874,12 +874,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-23 09:37:06</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -889,25 +884,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -917,382 +912,10 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-22 09:35:30</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C01000038</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>齿轮一</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>29</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-10-21 18:16:11</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>C01196394</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>输入轴</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CC091566</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>齿圈</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>磨齿</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-10-24 13:21:59</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-10-20 00:00:00</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>C01196057</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>高速轴1</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>子件</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>齿检仪检测</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-10-20 10:07:40</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>C01300536</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>大齿轮</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-10-23 18:27:54</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>C01310072</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>大齿圈</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-10-24 13:28:41</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>无断点</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1307,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1365,25 +988,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1393,32 +1016,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-25 10:31:12</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JC095136</t>
+          <t>CC090194</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>一级行星轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>风电项目（非远景）</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>清理喷丸</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1428,37 +1051,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-24 17:57:12</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-23 16:34:49</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196254</t>
+          <t>C01196402</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>低速齿轮轴46</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1468,28 +1086,33 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-24 19:56:51</t>
+          <t>2026-10-21 15:54:16</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01196403</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1503,29 +1126,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:30</t>
+          <t>2026-10-21 15:55:01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01300389</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1533,7 +1156,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1543,19 +1166,24 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-23 16:12:10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01196389</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>高速齿轮组38</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1568,7 +1196,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1578,19 +1206,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-24 13:15:22</t>
+          <t>2026-10-26 09:46:10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>C01196254</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>低速齿轮轴46</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1599,11 +1232,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1613,24 +1246,24 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-25 16:52:31</t>
+          <t>2026-10-24 19:56:51</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310074</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1638,7 +1271,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1648,29 +1281,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-25 07:17:52</t>
+          <t>2026-10-23 16:20:30</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-11-04 00:00:00</t>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01300339</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1678,7 +1311,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1688,37 +1321,37 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 19:38:15</t>
+          <t>2026-10-23 15:26:18</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>XZ00291</t>
+          <t>C01300533</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>行走齿轮箱（不含马达）</t>
+          <t>主齿轮组</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1728,47 +1361,392 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-22 15:00:25</t>
+          <t>2026-10-23 09:37:06</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>CC092697</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>齿轮</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>退磁</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:35:30</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-11-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C01300551</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CC091566</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>齿圈</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:21:59</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CC093021</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>大齿轮组件</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>动平衡</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:15:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C01196349</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-10-26 10:04:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C01300536</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CC090888</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>齿轮（右）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:38:15</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>XZ00291</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>行走齿轮箱（不含马达）</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>装配</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:00:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>C01000061</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>油泵齿轮</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>齿轮箱-高精</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D20" t="n">
         <v>2</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>调质</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>委外-完工</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>2026-10-23 16:36:38</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>2026-12-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>C01216011</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>中间级行星轮</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:14:17</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>无断点</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-26 15:09
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -427,6 +427,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,6 +476,11 @@
           <t>已开合格证</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>已开合格证时间</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -513,6 +519,11 @@
       <c r="I2" t="n">
         <v>7</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:22:08</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +562,11 @@
       <c r="I3" t="n">
         <v>2</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:43:39</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -594,6 +610,11 @@
       <c r="I4" t="n">
         <v>1</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-10-24 16:22:11</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -632,6 +653,11 @@
       <c r="I5" t="n">
         <v>1</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-10-24 16:22:11</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -675,6 +701,11 @@
       <c r="I6" t="n">
         <v>2</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-10-26 08:33:07</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -713,6 +744,11 @@
       <c r="I7" t="n">
         <v>29</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-10-23 13:14:42</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -756,6 +792,11 @@
       <c r="I8" t="n">
         <v>2</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-10-23 15:22:07</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -799,6 +840,11 @@
       <c r="I9" t="n">
         <v>3</v>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-10-25 16:01:37</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -842,6 +888,11 @@
       <c r="I10" t="n">
         <v>2</v>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-10-26 13:27:36</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -917,6 +968,11 @@
       </c>
       <c r="I12" t="n">
         <v>3</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2025-04-17 18:47:49</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-27 09:10
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -710,21 +710,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -738,27 +738,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-21 18:16:11</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-23 13:14:42</t>
+          <t>2026-10-26 15:09:34</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01000038</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿轮一</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -781,41 +781,36 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-21 18:13:17</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-23 15:22:07</t>
+          <t>2026-10-23 13:14:42</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01310072</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>大齿圈</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -829,45 +824,45 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-24 13:28:41</t>
+          <t>2026-10-23 13:00:35</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-25 16:01:37</t>
+          <t>2026-10-23 15:22:07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01310074</t>
+          <t>C01310072</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>大齿圈</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -877,45 +872,45 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-25 07:17:52</t>
+          <t>2026-10-24 13:28:41</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-11-04 00:00:00</t>
+          <t>2026-10-06 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-26 13:27:36</t>
+          <t>2026-10-25 16:01:37</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>C01310074</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>齿圈</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -925,51 +920,99 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-25 07:17:52</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-11-04 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-10-26 13:27:36</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>XY06110</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>输出行星轮</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>3</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>超精磨</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>2025-04-17 10:57:01</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="I13" t="n">
         <v>3</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>2025-04-17 18:47:49</t>
         </is>
@@ -986,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1044,17 +1087,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300548</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>内套II#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1062,34 +1105,39 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-26 14:34:36</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC090194</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1097,7 +1145,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1107,7 +1155,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-23 16:34:49</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
     </row>
@@ -1234,25 +1282,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196389</t>
+          <t>C01196254</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>高速齿轮组38</t>
+          <t>低速齿轮轴46</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1262,37 +1310,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-26 09:46:10</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-24 19:56:51</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196254</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>低速齿轮轴46</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1302,24 +1345,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-24 19:56:51</t>
+          <t>2026-10-23 16:20:26</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01350011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>偏置油缸齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1327,7 +1375,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1337,24 +1385,19 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:30</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-27 08:04:57</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300339</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1377,37 +1420,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 15:26:18</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-26 18:02:54</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300533</t>
+          <t>C01196349</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>主齿轮组</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1417,24 +1455,19 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-23 09:37:06</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-26 18:26:51</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CC092697</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1443,11 +1476,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1457,37 +1490,37 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-22 09:35:30</t>
+          <t>2026-10-23 18:27:54</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-11-01 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>CC090888</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1497,32 +1530,37 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-23 19:38:15</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CC091566</t>
+          <t>XZ00291</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>行走齿轮箱（不含马达）</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>装配</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1532,72 +1570,72 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-24 13:21:59</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-22 15:00:25</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-24 13:15:22</t>
+          <t>2026-10-23 16:36:38</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>C01216011</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>中间级行星轮</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1607,200 +1645,10 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-26 10:04:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>C01300536</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>大齿轮</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-10-23 18:27:54</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CC090888</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>齿轮（右）</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>摇臂钻2</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-10-23 19:38:15</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>XZ00291</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>行走齿轮箱（不含马达）</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>齿轮箱</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>装配</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-10-22 15:00:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>C01000061</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>油泵齿轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>齿轮箱-高精</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>调质</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-10-23 16:36:38</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-12-15 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
           <t>2026-09-14 16:14:17</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>无断点</t>
         </is>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-28 08:57
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -571,25 +571,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C07000134</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -599,20 +599,15 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-27 16:14:01</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-24 16:22:11</t>
+          <t>2026-10-27 19:39:51</t>
         </is>
       </c>
     </row>
@@ -637,7 +632,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -647,7 +642,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-24 15:45:06</t>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -662,12 +662,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300388</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -690,45 +690,40 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-24 18:29:46</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-24 15:45:06</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-26 08:33:07</t>
+          <t>2026-10-24 16:22:11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01300388</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -738,32 +733,37 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-24 18:29:46</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-26 15:09:34</t>
+          <t>2026-10-26 08:33:07</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01000038</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮一</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -781,7 +781,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-21 18:13:17</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-23 13:14:42</t>
+          <t>2026-10-26 15:09:34</t>
         </is>
       </c>
     </row>
@@ -844,25 +844,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01310072</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿圈</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -872,45 +872,40 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-24 13:28:41</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-06 00:00:00</t>
+          <t>2026-10-26 18:02:54</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-25 16:01:37</t>
+          <t>2026-10-27 16:18:32</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01310074</t>
+          <t>XY06109</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>齿圈</t>
+          <t>初级行星轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>滚齿2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -920,32 +915,22 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-25 07:17:52</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-11-04 00:00:00</t>
+          <t>2024-02-22 18:59:10</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2026-10-26 13:27:36</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>XY06110</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>输出行星轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -954,11 +939,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>超精磨</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -968,51 +953,13 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
         <v>3</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>3</v>
-      </c>
-      <c r="J13" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>2025-04-17 18:47:49</t>
         </is>
@@ -1029,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1162,25 +1109,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196402</t>
+          <t>C01300389</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1190,37 +1137,37 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-21 15:54:16</t>
+          <t>2026-10-23 16:12:10</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196403</t>
+          <t>C01300390</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1230,33 +1177,33 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-21 15:55:01</t>
+          <t>2026-10-27 09:45:56</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-26 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300389</t>
+          <t>C01196254</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>低速齿轮轴46</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1270,37 +1217,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23 16:12:10</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-24 19:56:51</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196254</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>低速齿轮轴46</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1310,32 +1252,37 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-24 19:56:51</t>
+          <t>2026-10-23 16:20:26</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01350011</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>偏置油缸齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1345,24 +1292,19 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:26</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-27 14:00:02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01350011</t>
+          <t>C01196349</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>偏置油缸齿轮</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1371,11 +1313,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1385,24 +1327,24 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-27 08:04:57</t>
+          <t>2026-10-27 16:20:52</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1410,7 +1352,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1420,32 +1362,37 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-26 18:02:54</t>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>CC090888</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1455,139 +1402,144 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-26 18:26:51</t>
+          <t>2026-10-23 19:38:15</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C07106019</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>低速输出轴</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C01196458</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23 19:38:15</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-12-04 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XZ00291</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>行走齿轮箱（不含马达）</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-22 15:00:25</t>
+          <t>2026-10-23 16:36:38</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01000061</t>
+          <t>C01196092</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>油泵齿轮</t>
+          <t>二级齿轮轴</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1595,62 +1547,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>调质</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-23 16:36:38</t>
+          <t>2026-10-27 10:39:05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-12-15 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>C01216011</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>中间级行星轮</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-09-14 16:14:17</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>无断点</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1769,25 +1681,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C07000134</t>
+          <t>C01300321</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>被动同步齿轮组</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>外圆磨2</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1797,29 +1709,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-20 19:18:57</t>
+          <t>2026-10-27 12:43:57</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01300492</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>被动同步齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -1827,7 +1744,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1837,42 +1754,37 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-17 11:31:39</t>
+          <t>2026-10-28 05:45:45</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196092</t>
+          <t>C01196231</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>二级齿轮轴</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>加工中心3</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1882,17 +1794,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-25 23:21:25</t>
+          <t>2026-10-28 02:35:36</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-29 08:41
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -513,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-25 10:31:12</t>
+          <t>2026-10-28 17:26:28</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-22 14:41:55</t>
+          <t>2026-10-28 13:39:00</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -796,25 +796,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01350011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>偏置油缸齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -824,37 +824,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-27 14:00:02</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-23 15:22:07</t>
+          <t>2026-10-28 14:04:12</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -862,7 +857,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -872,40 +867,45 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-26 18:02:54</t>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 16:18:32</t>
+          <t>2026-10-23 15:22:07</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>XY06109</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>初级行星轮</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>滚齿2</t>
+          <t>动平衡</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -915,51 +915,142 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2024-02-22 18:59:10</t>
+          <t>2026-10-26 18:02:54</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>1</v>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-10-27 16:18:32</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>CC090888</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>齿轮（右）</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>油气</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>摇臂钻2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:38:15</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>7</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>XY06110</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>输出行星轮</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>3</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>超精磨</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>2025-04-17 10:57:01</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="I14" t="n">
         <v>3</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>2025-04-17 18:47:49</t>
         </is>
@@ -976,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1189,25 +1280,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196254</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>低速齿轮轴46</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1217,19 +1308,24 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-24 19:56:51</t>
+          <t>2026-10-23 16:20:26</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01300321</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>被动同步齿轮组</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1252,37 +1348,37 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:26</t>
+          <t>2026-10-28 18:31:08</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01350011</t>
+          <t>C01300492</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>偏置油缸齿轮</t>
+          <t>被动同步齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1292,7 +1388,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-27 14:00:02</t>
+          <t>2026-10-28 18:15:01</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1414,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1327,7 +1428,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-27 16:20:52</t>
+          <t>2026-10-28 15:49:47</t>
         </is>
       </c>
     </row>
@@ -1374,57 +1475,52 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C07106019</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>低速输出轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-23 19:38:15</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C07106019</t>
+          <t>C01196458</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>低速输出轴</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1445,16 +1541,21 @@
           <t>2026-10-27 17:33:13</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-12-04 00:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01196458</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1463,11 +1564,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1477,29 +1578,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
+          <t>2026-10-23 16:36:38</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-12-04 00:00:00</t>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01000061</t>
+          <t>C01196092</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>油泵齿轮</t>
+          <t>二级齿轮轴</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1507,60 +1608,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>调质</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-23 16:36:38</t>
+          <t>2026-10-27 10:39:05</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-12-15 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>C01196092</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>二级齿轮轴</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-10-27 10:39:05</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
         <is>
           <t>2026-10-10 00:00:00</t>
         </is>
@@ -1641,17 +1702,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01196231</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1659,7 +1720,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1669,7 +1730,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-23 15:01:14</t>
+          <t>2026-10-28 02:35:36</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1681,17 +1742,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300321</t>
+          <t>CC090707</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>被动同步齿轮组</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1709,42 +1770,42 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-27 12:43:57</t>
+          <t>2026-10-28 16:23:47</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-11-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300492</t>
+          <t>CC090493</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>被动同步齿轮</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>加工中心2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1754,29 +1815,29 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-28 05:45:45</t>
+          <t>2026-10-28 15:05:47</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01196231</t>
+          <t>C01300543</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>被动齿轮组件</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -1794,7 +1855,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-28 02:35:36</t>
+          <t>2026-10-29 06:42:53</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-30 08:28
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -485,25 +485,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,40 +513,45 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-28 17:26:28</t>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-26 14:22:08</t>
+          <t>2026-10-24 16:22:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01300388</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -556,7 +561,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-28 13:39:00</t>
+          <t>2026-10-24 18:29:46</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -564,14 +574,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-24 18:43:39</t>
+          <t>2026-10-26 08:33:07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C07000134</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -581,7 +591,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -599,7 +609,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-27 16:14:01</t>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -607,32 +622,32 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:39:51</t>
+          <t>2026-10-23 15:22:07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>CC090888</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>摇臂钻2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -642,417 +657,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-23 19:38:15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-24 16:22:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>C01300387</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>齿轮M</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>酸蚀检验</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-24 15:45:06</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-10-24 16:22:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>C01300388</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>齿轮J</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>酸蚀检验</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-10-24 18:29:46</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2026-10-26 08:33:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>C01300551</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>大齿轮</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>子件</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-10-23 14:48:27</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2026-10-26 15:09:34</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>C01350011</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>偏置油缸齿轮</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>子件</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>加工中心</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2026-10-27 14:00:02</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2026-10-28 14:04:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>C01196394</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>输入轴</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>散单</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-10-23 15:22:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CC093021</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>大齿轮组件</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>高精高速</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>动平衡</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-10-26 18:02:54</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2026-10-27 16:18:32</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CC090888</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>齿轮（右）</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>油气</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>摇臂钻2</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-23 19:38:15</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>7</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
           <t>2026-10-28 18:14:13</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2025-04-17 18:47:49</t>
         </is>
       </c>
     </row>
@@ -1067,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1165,17 +783,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300550</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1183,7 +801,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1193,19 +811,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-29 16:34:17</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300389</t>
+          <t>C01310071</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>外套#</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1228,7 +851,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-23 16:12:10</t>
+          <t>2026-10-29 12:45:56</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1240,17 +863,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300390</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -1258,7 +881,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1268,37 +891,32 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-27 09:45:56</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-28 17:26:28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1308,24 +926,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:26</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-29 14:32:16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300321</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>被动同步齿轮组</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1338,7 +951,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1348,24 +961,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-28 18:31:08</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-24 15:45:06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300492</t>
+          <t>C01300390</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>被动同步齿轮</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1374,11 +982,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1388,37 +996,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-28 18:15:01</t>
+          <t>2026-10-27 09:45:56</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1428,24 +1036,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-28 15:49:47</t>
+          <t>2026-10-23 16:20:26</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C01300321</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>被动同步齿轮组</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1463,64 +1076,69 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
+          <t>2026-10-28 18:31:08</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C07106019</t>
+          <t>C01300492</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>低速输出轴</t>
+          <t>被动同步齿轮</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
+          <t>2026-10-28 18:15:01</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01196458</t>
+          <t>CC090493</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1528,79 +1146,74 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-12-04 00:00:00</t>
+          <t>2026-10-29 18:49:52</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01000061</t>
+          <t>C01390025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>油泵齿轮</t>
+          <t>主小齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>调质</t>
+          <t>打标</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23 16:36:38</t>
+          <t>2026-10-29 19:19:58</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-12-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01196092</t>
+          <t>CC093021</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>二级齿轮轴</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1608,22 +1221,287 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>动平衡</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:02:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C01196058</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>高速轴组件1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>外圆磨</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-10-29 19:50:54</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C01300536</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C01196458</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>齿轮箱-高精</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>锻造</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:33:13</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-12-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C01000061</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>油泵齿轮</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>齿轮箱-高精</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>调质</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:36:38</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-12-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01196092</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>二级齿轮轴</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>2026-10-27 10:39:05</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1716,7 +1594,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1730,7 +1608,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-28 02:35:36</t>
+          <t>2026-10-29 19:46:05</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1787,12 +1665,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CC090493</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1801,11 +1679,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>加工中心2</t>
+          <t>外圆磨2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1815,52 +1693,197 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-28 15:05:47</t>
+          <t>2026-10-29 14:50:55</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>C01300542</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>主动齿轮</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:36:29</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>C01300543</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>被动齿轮组件</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>散单</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>磨齿</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-29 06:42:53</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-29 13:00:34</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C01196091</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>三级齿轮轴</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>加工中心2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-10-29 17:40:27</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C01000060</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>输入大齿轮</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:14:26</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-30 17:46
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01310071</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>外套#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
+          <t>2026-10-29 12:45:56</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -522,36 +522,36 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-24 16:22:11</t>
+          <t>2026-10-29 15:02:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300388</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -561,41 +561,36 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-24 18:29:46</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-29 14:32:16</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-26 08:33:07</t>
+          <t>2026-10-29 18:29:21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -609,37 +604,32 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-28 17:26:28</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-23 15:22:07</t>
+          <t>2026-10-29 18:56:29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CC090888</t>
+          <t>C07000134</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -647,7 +637,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>摇臂钻2</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -657,20 +647,455 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-23 19:38:15</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-27 16:14:01</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-28 18:14:13</t>
+          <t>2026-10-27 19:39:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C01300387</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>齿轮M</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>齿检仪检测</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-10-24 16:22:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C01300387</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>齿轮M</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>酸蚀检验</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-10-24 15:45:06</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-10-24 16:22:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C01300388</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>齿轮J</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>高精高速</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>酸蚀检验</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:29:46</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-10-26 08:33:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CC090493</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>齿轮</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>退磁</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:49:52</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:56:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C01300551</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:48:27</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:09:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C01350011</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>偏置油缸齿轮</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>加工中心</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-10-27 14:00:02</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-10-28 14:04:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C01196394</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>输入轴</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>散单</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-10-23 15:22:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C01196349</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>22</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>磨齿</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:49:47</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>22</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-10-30 14:00:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>XY06109</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>初级行星轮</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>滚齿2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2024-02-22 18:59:10</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>XY06110</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>输出行星轮</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>超精磨</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2025-04-17 10:57:01</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2025-04-17 18:47:49</t>
         </is>
       </c>
     </row>
@@ -685,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -823,17 +1248,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01310071</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>外套#</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -841,7 +1266,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -851,29 +1276,24 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-29 12:45:56</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01300390</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮J</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -881,7 +1301,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -891,32 +1311,37 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-28 17:26:28</t>
+          <t>2026-10-27 09:45:56</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01196387</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>低速齿轮组45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -926,24 +1351,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-29 14:32:16</t>
+          <t>2026-10-23 16:20:26</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C01390025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>主小齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -951,7 +1381,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>打标</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -961,19 +1391,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-24 15:45:06</t>
+          <t>2026-10-29 19:19:58</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300390</t>
+          <t>C01196058</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>高速轴组件1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -986,7 +1421,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -996,33 +1431,33 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-27 09:45:56</t>
+          <t>2026-10-29 19:50:54</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01196387</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>低速齿轮组45</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1036,29 +1471,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 16:20:26</t>
+          <t>2026-10-23 18:27:54</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-25 00:00:00</t>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300321</t>
+          <t>C14006243</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>被动同步齿轮组</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1066,7 +1501,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1076,37 +1511,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-28 18:31:08</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-30 14:16:32</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01300492</t>
+          <t>C14006243</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>被动同步齿轮</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1116,29 +1546,24 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-28 18:15:01</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-31 00:00:00</t>
+          <t>2026-10-30 14:16:32</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CC090493</t>
+          <t>C07106019</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>低速输出轴</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1146,117 +1571,122 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-29 18:49:52</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01390025</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>主小齿轮</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>打标</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-29 19:19:58</t>
+          <t>2026-10-23 16:36:38</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CC093021</t>
+          <t>C01196458</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>动平衡</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-26 18:02:54</t>
+          <t>2026-10-27 17:33:13</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-12-04 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01196058</t>
+          <t>C01196091</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>高速轴组件1</t>
+          <t>三级齿轮轴</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1266,29 +1696,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-29 19:50:54</t>
+          <t>2026-10-30 09:43:36</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C01196092</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>二级齿轮轴</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1306,202 +1736,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
+          <t>2026-10-27 10:39:05</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>C01196458</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>高速齿轮轴</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>齿轮箱-高精</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>锻造</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-10-27 17:33:13</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2026-12-04 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>C01000061</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>油泵齿轮</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>齿轮箱-高精</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>调质</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>委外-完工</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-10-23 16:36:38</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-12-15 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>C01196092</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>二级齿轮轴</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-10-27 10:39:05</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
           <t>2026-10-10 00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>XY06109</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>初级行星轮</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>滚齿2</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2024-02-22 18:59:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>XY06110</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>输出行星轮</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>齿轮箱-普通</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>超精磨</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2025-04-17 10:57:01</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1834,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1608,7 +1848,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:46:05</t>
+          <t>2026-10-30 11:03:53</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1800,45 +2040,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01196091</t>
+          <t>C07000069</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>三级齿轮轴</t>
+          <t>轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>加工中心2</t>
+          <t>外圆磨2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-29 17:40:27</t>
+          <t>2026-10-29 16:01:35</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-31 07:52
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01310071</t>
+          <t>C01300550</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>外套#</t>
+          <t>大齿轮组件</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:45:56</t>
+          <t>2026-10-29 16:34:17</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -526,32 +526,32 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:02:58</t>
+          <t>2026-10-30 16:40:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01310071</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>外套#</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -561,27 +561,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-29 14:32:16</t>
+          <t>2026-10-29 12:45:56</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-29 18:29:21</t>
+          <t>2026-10-29 15:02:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -590,11 +595,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -604,36 +609,41 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-28 17:26:28</t>
+          <t>2026-10-30 15:15:51</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-29 18:56:29</t>
+          <t>2026-10-29 18:29:21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C07000134</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -647,40 +657,40 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-27 16:14:01</t>
+          <t>2026-10-28 17:26:28</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:39:51</t>
+          <t>2026-10-29 18:56:29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>C07000134</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -690,12 +700,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-27 16:14:01</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -703,7 +708,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-24 16:22:11</t>
+          <t>2026-10-27 19:39:51</t>
         </is>
       </c>
     </row>
@@ -728,7 +733,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -738,40 +743,40 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-24 15:45:06</t>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2026-10-24 16:22:11</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01300388</t>
+          <t>CC090493</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮J</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>酸蚀检验</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -781,37 +786,32 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-24 18:29:46</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-29 18:49:52</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-26 08:33:07</t>
+          <t>2026-10-29 18:56:43</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CC090493</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -819,7 +819,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-29 18:49:52</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -837,19 +837,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-29 18:56:43</t>
+          <t>2026-10-26 15:09:34</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01350011</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>偏置油缸齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -858,11 +858,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -872,40 +872,40 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-27 14:00:02</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-26 15:09:34</t>
+          <t>2026-10-28 14:04:12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01350011</t>
+          <t>C01196393</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>偏置油缸齿轮</t>
+          <t>涡轮轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -915,15 +915,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-27 14:00:02</t>
+          <t>2026-10-30 13:40:03</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-28 14:04:12</t>
+          <t>2026-10-30 13:45:56</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1208,17 +1213,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01300550</t>
+          <t>C14006233</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>三级推力盘转接套</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1226,7 +1231,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>精车2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1236,37 +1241,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-29 16:34:17</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-09-17 05:04:50</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>XY01124</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>扭力管</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>酸蚀检验</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-30 18:42:02</t>
         </is>
       </c>
     </row>
@@ -1483,12 +1483,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C14006243</t>
+          <t>C14006242</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>高速推力盘</t>
+          <t>低速推力盘</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-30 14:16:32</t>
+          <t>2026-10-30 15:29:51</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C07106019</t>
+          <t>C14006243</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>低速输出轴</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1567,46 +1567,46 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
+          <t>2026-10-30 14:16:32</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01000061</t>
+          <t>C07106019</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>油泵齿轮</t>
+          <t>低速输出轴</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>调质</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1616,24 +1616,19 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23 16:36:38</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-12-15 00:00:00</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01196458</t>
+          <t>C01000061</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>油泵齿轮</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1642,11 +1637,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1656,64 +1651,64 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
+          <t>2026-10-23 16:36:38</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-12-04 00:00:00</t>
+          <t>2026-12-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01196091</t>
+          <t>C01196458</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>三级齿轮轴</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>齿轮箱-高精</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-30 09:43:36</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-12-04 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01196092</t>
+          <t>C01196091</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>二级齿轮轴</t>
+          <t>三级齿轮轴</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1736,10 +1731,50 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>2026-10-30 09:43:36</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C01196092</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>二级齿轮轴</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>2026-10-27 10:39:05</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>2026-10-10 00:00:00</t>
         </is>
@@ -1834,7 +1869,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1848,7 +1883,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-30 11:03:53</t>
+          <t>2026-10-30 19:26:03</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1905,12 +1940,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01300542</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>主动齿轮</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1923,7 +1958,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>外圆磨2</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1933,7 +1968,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-29 14:50:55</t>
+          <t>2026-10-29 18:36:29</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1950,12 +1985,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300542</t>
+          <t>C01300543</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>主动齿轮</t>
+          <t>被动齿轮组件</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1978,7 +2013,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-29 18:36:29</t>
+          <t>2026-10-29 13:00:34</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1995,70 +2030,65 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C01300543</t>
+          <t>C07000069</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>被动齿轮组件</t>
+          <t>轴</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-29 13:00:34</t>
+          <t>2026-10-29 16:01:35</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C07000069</t>
+          <t>C01000060</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轴</t>
+          <t>输入大齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>齿轮箱-普通</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>外圆磨2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2068,24 +2098,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-29 16:01:35</t>
+          <t>2026-10-29 16:14:26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01000060</t>
+          <t>C01196093</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>输入大齿轮</t>
+          <t>主轴</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2094,31 +2129,26 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-29 16:14:26</t>
+          <t>2026-10-30 23:20:14</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-11-15 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update feifeng-wangong-xlsx 2026-10-31 14:02
</commit_message>
<xml_diff>
--- a/feifeng-wangong.xlsx
+++ b/feifeng-wangong.xlsx
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300550</t>
+          <t>C01310071</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>大齿轮组件</t>
+          <t>外套#</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:34:17</t>
+          <t>2026-10-29 12:45:56</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -526,32 +526,32 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:40:00</t>
+          <t>2026-10-29 15:02:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C01310071</t>
+          <t>C01196162</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>外套#</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>油气</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -561,32 +561,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-29 12:45:56</t>
+          <t>2026-10-31 13:32:55</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-29 15:02:58</t>
+          <t>2026-10-29 18:29:21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01196162</t>
+          <t>C01300254</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>齿轮（右）</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -595,11 +595,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -609,41 +609,36 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-30 15:15:51</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-28 17:26:28</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-29 18:29:21</t>
+          <t>2026-10-29 18:56:29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300254</t>
+          <t>C07000134</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>齿轮（右）</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>油气</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -657,40 +652,40 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-28 17:26:28</t>
+          <t>2026-10-27 16:14:01</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-29 18:56:29</t>
+          <t>2026-10-27 19:39:51</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C07000134</t>
+          <t>C01300387</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>齿轮M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>齿检仪检测</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -700,32 +695,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-27 16:14:01</t>
+          <t>2026-10-13 15:21:27</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-10-27 19:39:51</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01300387</t>
+          <t>CC090493</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>齿轮M</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -733,7 +728,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>齿检仪检测</t>
+          <t>退磁</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -743,32 +738,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13 15:21:27</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-29 18:49:52</t>
         </is>
       </c>
       <c r="I7" t="n">
         <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:56:43</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CC090493</t>
+          <t>C01300551</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -776,7 +771,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>退磁</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -786,7 +781,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-29 18:49:52</t>
+          <t>2026-10-23 14:48:27</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -794,19 +789,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-29 18:56:43</t>
+          <t>2026-10-26 15:09:34</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300551</t>
+          <t>C01350011</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>偏置油缸齿轮</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -815,11 +810,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>加工中心</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -829,40 +824,40 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 14:48:27</t>
+          <t>2026-10-27 14:00:02</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-26 15:09:34</t>
+          <t>2026-10-28 14:04:12</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C01350011</t>
+          <t>C01196394</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>偏置油缸齿轮</t>
+          <t>输入轴</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>加工中心</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -872,40 +867,45 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-27 14:00:02</t>
+          <t>2026-10-23 13:00:35</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-28 14:04:12</t>
+          <t>2026-10-23 15:22:07</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C01196393</t>
+          <t>C01196349</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>涡轮轴</t>
+          <t>高速齿轮轴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -915,37 +915,32 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-30 13:40:03</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-28 15:49:47</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-30 13:45:56</t>
+          <t>2026-10-30 14:00:06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C01196394</t>
+          <t>C14006243</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>输入轴</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -953,7 +948,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -963,12 +958,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-23 13:00:35</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-30 14:16:32</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -976,19 +966,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-23 15:22:07</t>
+          <t>2026-10-31 13:49:36</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C01196349</t>
+          <t>C14006243</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -997,11 +987,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>磨内孔</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1011,15 +1001,15 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-28 15:49:47</t>
+          <t>2026-10-30 14:16:32</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-30 14:00:06</t>
+          <t>2026-10-31 13:49:36</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1173,12 +1163,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01300548</t>
+          <t>C01196397</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>内套II#</t>
+          <t>小齿轮组</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1191,17 +1181,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-26 14:34:36</t>
+          <t>2026-10-31 13:13:10</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1213,17 +1203,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C14006233</t>
+          <t>C01300548</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>三级推力盘转接套</t>
+          <t>内套II#</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1231,17 +1221,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>精车2</t>
+          <t>线切割</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 05:04:50</t>
+          <t>2026-10-26 14:34:36</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
         </is>
       </c>
     </row>
@@ -1363,25 +1358,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01390025</t>
+          <t>C01196231</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>主小齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>打标</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1391,29 +1386,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-29 19:19:58</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-31 10:39:46</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C01196058</t>
+          <t>C01390025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>高速轴组件1</t>
+          <t>主小齿轮</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>高精高速</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1421,7 +1411,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>外圆磨</t>
+          <t>打标</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1431,37 +1421,37 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-29 19:50:54</t>
+          <t>2026-10-29 19:19:58</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-20 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C01300536</t>
+          <t>C01196058</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>大齿轮</t>
+          <t>高速轴组件1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1471,37 +1461,37 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-23 18:27:54</t>
+          <t>2026-10-29 19:50:54</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-07 00:00:00</t>
+          <t>2026-10-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C14006242</t>
+          <t>C01300536</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>低速推力盘</t>
+          <t>大齿轮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1511,19 +1501,24 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-30 15:29:51</t>
+          <t>2026-10-23 18:27:54</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C14006243</t>
+          <t>C14006242</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>高速推力盘</t>
+          <t>低速推力盘</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1532,7 +1527,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1546,19 +1541,19 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-30 14:16:32</t>
+          <t>2026-10-30 15:29:51</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C14006243</t>
+          <t>C07106019</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>高速推力盘</t>
+          <t>低速输出轴</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1567,33 +1562,33 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>磨内孔</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-30 14:16:32</t>
+          <t>2026-10-27 17:33:13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C07106019</t>
+          <t>C01196450</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>低速输出轴</t>
+          <t>低速齿轮轴</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1602,7 +1597,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1616,32 +1611,32 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
+          <t>2026-10-24 15:18:45</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C01000061</t>
+          <t>C14006273</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>油泵齿轮</t>
+          <t>低速推力盘</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>调质</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1651,37 +1646,32 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-10-23 16:36:38</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-12-15 00:00:00</t>
+          <t>2026-10-24 15:19:18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C01196458</t>
+          <t>C14006274</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>高速齿轮轴</t>
+          <t>低速推力盘套</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>齿轮箱-高精</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>锻造</t>
+          <t>调质</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1691,90 +1681,340 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-10-27 17:33:13</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-12-04 00:00:00</t>
+          <t>2026-10-23 16:37:52</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C01196091</t>
+          <t>C14006275</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>三级齿轮轴</t>
+          <t>高速推力盘</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>锻造</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>自制-完工</t>
+          <t>委外-完工</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-10-30 09:43:36</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-10-10 00:00:00</t>
+          <t>2026-10-24 15:20:50</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>C14006276</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>高速推力盘套</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>调质</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:38:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C01196451</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>锻造</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-10-24 15:19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01300578</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>大齿轮</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>调质</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-10-30 15:47:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>C01196452</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>输入齿轮轴</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>调质</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:37:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>C01000061</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>油泵齿轮</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>齿轮箱-高精</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>调质</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:36:38</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-12-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C01196458</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>高速齿轮轴</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>齿轮箱-高精</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>锻造</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:33:13</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-12-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>C01196091</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>三级齿轮轴</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-10-30 09:43:36</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>C01196092</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>二级齿轮轴</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D24" t="n">
         <v>2</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>2026-10-27 10:39:05</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>2026-10-10 00:00:00</t>
         </is>
@@ -1791,7 +2031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1855,12 +2095,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01196231</t>
+          <t>C01196255</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>齿轮轴</t>
+          <t>低速齿轮组46</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1869,11 +2109,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1883,7 +2123,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:26:03</t>
+          <t>2026-10-31 10:29:30</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1895,17 +2135,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CC090707</t>
+          <t>C01196231</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>齿轮</t>
+          <t>齿轮轴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>高精高速</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1923,42 +2163,37 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-28 16:23:47</t>
+          <t>2026-10-30 11:03:53</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>磁粉探伤-退磁</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-11-25 00:00:00</t>
+          <t>磁粉探伤</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C01300542</t>
+          <t>C07000106</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>主动齿轮</t>
+          <t>轴</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>散单</t>
+          <t>子件</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>磨齿</t>
+          <t>外圆磨2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1968,29 +2203,24 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-29 18:36:29</t>
+          <t>2026-10-31 12:31:33</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C01300543</t>
+          <t>CC090707</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>被动齿轮组件</t>
+          <t>齿轮</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1999,7 +2229,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2013,92 +2243,97 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-29 13:00:34</t>
+          <t>2026-10-28 16:23:47</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>磁粉探伤</t>
+          <t>磁粉探伤-退磁</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-11-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C07000069</t>
+          <t>C01300542</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>轴</t>
+          <t>主动齿轮</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>子件</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>外圆磨2</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-29 16:01:35</t>
+          <t>2026-10-29 18:36:29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C01000060</t>
+          <t>C01300543</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>输入大齿轮</t>
+          <t>被动齿轮组件</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>齿轮箱-普通</t>
+          <t>散单</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>线切割</t>
+          <t>磨齿</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>委外-完工</t>
+          <t>自制-完工</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-29 16:14:26</t>
+          <t>2026-10-29 13:00:34</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2108,45 +2343,130 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-11-15 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>C07000069</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>轴</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>子件</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>外圆磨2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:01:35</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C01000060</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>输入大齿轮</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>齿轮箱-普通</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>线切割</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>委外-完工</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:14:26</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>磁粉探伤</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-11-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>C01196093</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>主轴</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>齿轮箱-普通</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>齿检仪检测</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>自制-完工</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>自制-完工</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>2026-10-30 23:20:14</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>磁粉探伤</t>
         </is>

</xml_diff>